<commit_message>
day 1 final updates and day 2 setup
Basic excel operations and formulas
</commit_message>
<xml_diff>
--- a/Day_01__excel_introduction.xlsx
+++ b/Day_01__excel_introduction.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f5c7b832c0e5f38/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f5c7b832c0e5f38/Documents/My projects/100-days-of-data-repository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{166FA2C6-E154-400C-9B96-16E123C2541D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{166FA2C6-E154-400C-9B96-16E123C2541D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90A55DF0-6F80-4043-89EF-20953798E480}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7A30BAB1-110D-4B5F-BCCD-737F928A097E}"/>
+    <workbookView xWindow="8630" yWindow="380" windowWidth="10570" windowHeight="7270" xr2:uid="{7A30BAB1-110D-4B5F-BCCD-737F928A097E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>NAME</t>
   </si>
@@ -106,6 +106,21 @@
   </si>
   <si>
     <t>average salary of sales</t>
+  </si>
+  <si>
+    <t>of finance</t>
+  </si>
+  <si>
+    <t>average salary for procurement</t>
+  </si>
+  <si>
+    <t>sum of finance</t>
+  </si>
+  <si>
+    <t>sum of sales</t>
+  </si>
+  <si>
+    <t>sum of procurement</t>
   </si>
 </sst>
 </file>
@@ -458,14 +473,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F186B07-6137-4A2E-B16A-6D2DC6883CC9}">
-  <dimension ref="A2:D17"/>
+  <dimension ref="A2:D23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.6328125" customWidth="1"/>
-    <col min="2" max="2" width="11.6328125" customWidth="1"/>
+    <col min="2" max="2" width="20.6328125" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -476,7 +492,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -487,7 +503,7 @@
         <v>60270</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -498,7 +514,7 @@
         <v>39627</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -509,7 +525,7 @@
         <v>29727</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -520,7 +536,7 @@
         <v>93668</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -531,7 +547,7 @@
         <v>134000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -542,7 +558,7 @@
         <v>34808</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -553,7 +569,7 @@
         <v>134468</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -564,7 +580,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>16</v>
       </c>
@@ -573,58 +589,113 @@
         <v>571568</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="1">
+        <f>SUMIFS(C3:C10,B3:B10,"finance")</f>
+        <v>223997</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="1">
+        <f>SUMIFS(C3:C10,B3:B10,"sales")</f>
+        <v>302571</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="1">
+        <f>SUMIFS(C3:C10,B3:B10,"procurement")</f>
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C15" s="1"/>
+      <c r="D15" s="1">
+        <f>SUM(C12+C13+C14)</f>
+        <v>571568</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C16" s="1">
         <f>AVERAGE(C3:C10)</f>
         <v>71446</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
         <v>18</v>
       </c>
-      <c r="C13">
+      <c r="C17">
         <f>COUNT(C3:C10)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="C14">
+      <c r="C18">
         <f>COUNTA(C3:C10)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C19" s="1">
         <f>MIN(C3:C10)</f>
         <v>29727</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C20" s="1">
         <f>MAX(C3:C10)</f>
         <v>134468</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" t="s">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
         <v>22</v>
       </c>
-      <c r="D17">
+      <c r="D21">
         <f>AVERAGEIFS(C3:C10,B3:B10,"Sales")</f>
         <v>75642.75</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22">
+        <f>AVERAGEIFS(C3:C10,B3:B10,"finance")</f>
+        <v>74665.666666666672</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23">
+        <f>AVERAGEIFS(C3:C10,B3:B10,"procurement")</f>
+        <v>45000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>